<commit_message>
Add Telugu and bilingual (English + Telugu) reminder messages
- Batch message language on the Review step: English, Telugu, or
  English + Telugu in one message; both templates editable with live preview
- Optional "Language" Excel column (English / Telugu / Both) overrides the
  batch language per customer; invalid values are reported in validation
- Default Telugu template, editable under Settings → Message Template
- Language stored per record, shown in the recipients table and Excel export
- WhatsApp provider picks the matching approved template per language
  (WHATSAPP_TEMPLATE_NAME_TE / _LANGUAGE_TE, WHATSAPP_TEMPLATE_NAME_BOTH ...)
- Migration adds language columns; existing batches default to English
- Tests for rendering, Excel column, per-customer override, provider template
  selection and template permissions

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017LPjQcuJmn3Av7CcoYMBLq
</commit_message>
<xml_diff>
--- a/templates/bulk-whatsapp-reminder-template.xlsx
+++ b/templates/bulk-whatsapp-reminder-template.xlsx
@@ -73,12 +73,19 @@
         </r>
       </text>
     </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <t>Optional</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="33">
   <si>
     <t>Customer Name</t>
   </si>
@@ -104,6 +111,9 @@
     <t>Custom Message</t>
   </si>
   <si>
+    <t>Language</t>
+  </si>
+  <si>
     <t>Ravi Kumar</t>
   </si>
   <si>
@@ -125,6 +135,9 @@
     <t>SAMPLE ROW – delete this row before uploading (it is ignored on import)</t>
   </si>
   <si>
+    <t>English</t>
+  </si>
+  <si>
     <t>Column</t>
   </si>
   <si>
@@ -162,6 +175,9 @@
   </si>
   <si>
     <t>Optional extra line added to the message.</t>
+  </si>
+  <si>
+    <t>Optional. English, Telugu or Both (English + Telugu in one message). Empty = the language chosen for the batch.</t>
   </si>
   <si>
     <t/>
@@ -567,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" style="1" customWidth="1"/>
@@ -576,9 +592,10 @@
     <col min="5" max="5" width="21" style="1" customWidth="1"/>
     <col min="6" max="7" width="24" style="1" customWidth="1"/>
     <col min="8" max="8" width="20" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -603,31 +620,37 @@
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="I1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" s="6">
         <v>5000</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -639,7 +662,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -649,13 +672,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -663,10 +686,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -674,10 +697,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -685,10 +708,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -696,10 +719,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -707,10 +730,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -718,10 +741,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -729,10 +752,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -740,21 +763,32 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>